<commit_message>
Produzione Fase 1 in produzione; DP13 approvata (da confermare con l'agronomo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Domande-cantina.xlsx
+++ b/docs/Domande-cantina.xlsx
@@ -678,7 +678,7 @@
     <t>Chiesta</t>
   </si>
   <si>
-    <t>25/09/2026: Dante lo chiede all'agronomo (è la decisione DP13).</t>
+    <t>25/09/2026: Dante approva la proposta (anno solare); resta da confermare con l'agronomo. Nel software è la soglia «Periodo delle applicazioni massime».</t>
   </si>
   <si>
     <t>VIG-12</t>
@@ -2169,10 +2169,10 @@
     <t>Per il vigneto: anno di vendemmia e anno solare; la campagna 1/8–31/7 per cantina e registro</t>
   </si>
   <si>
-    <t>Aperta: Dante la chiede all'agronomo</t>
-  </si>
-  <si>
-    <t>Domanda VIG-11.</t>
+    <t>Approvata da Dante: anno solare per le applicazioni massime, annata di vendemmia per i costi di vigneto</t>
+  </si>
+  <si>
+    <t>Da confermare con l'agronomo (VIG-11). Nel software è una soglia modificabile.</t>
   </si>
   <si>
     <t>DP14</t>

</xml_diff>